<commit_message>
Cloud hosting: vendor SyGMa, in-process engine, Streamlit Cloud config
</commit_message>
<xml_diff>
--- a/benchmark/results/mass_accuracy_table.xlsx
+++ b/benchmark/results/mass_accuracy_table.xlsx
@@ -49,7 +49,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F7FF"/>
+        <fgColor rgb="00EBF4FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -801,34 +801,34 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Oseltamivir</t>
+          <t>Naproxen</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>C16H28N2O4</t>
+          <t>C14H14O3</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>312.2049</v>
+        <v>230.0943</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>300.2049</v>
+        <v>230.0943</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>-38436.296</v>
+        <v>0</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>313.2122</v>
+        <v>231.1016</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>301.2122</v>
+        <v>231.1016</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>-38312.684</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -843,25 +843,25 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>558.248</v>
+        <v>558.253</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>558.253</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>8.957000000000001</v>
+        <v>0</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>559.2553</v>
+        <v>559.2603</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>559.2603</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>8.94</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1398,55 +1398,55 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Oseltamivir</t>
+          <t>Naproxen</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C16H28N2O4</t>
+          <t>C14H14O3</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>medium (312 Da)</t>
+          <t>medium (230 Da)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>312.2049</v>
+        <v>230.0943</v>
       </c>
       <c r="E10" t="n">
-        <v>300.2049</v>
+        <v>230.0943</v>
       </c>
       <c r="F10" t="n">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>-38436.296</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>313.2122</v>
+        <v>231.1016</v>
       </c>
       <c r="I10" t="n">
-        <v>301.2122</v>
+        <v>231.1016</v>
       </c>
       <c r="J10" t="n">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>-38312.684</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>311.1976</v>
+        <v>229.087</v>
       </c>
       <c r="M10" t="n">
-        <v>299.1976</v>
+        <v>229.087</v>
       </c>
       <c r="N10" t="n">
-        <v>-38560.709</v>
+        <v>0</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>NIST, PubChem CID 65028</t>
+          <t>NIST, PubChem CID 156391</t>
         </is>
       </c>
     </row>
@@ -1467,37 +1467,37 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>558.248</v>
+        <v>558.253</v>
       </c>
       <c r="E11" t="n">
         <v>558.253</v>
       </c>
       <c r="F11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>8.957000000000001</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>559.2553</v>
+        <v>559.2603</v>
       </c>
       <c r="I11" t="n">
         <v>559.2603</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>8.94</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>557.2406999999999</v>
+        <v>557.2457000000001</v>
       </c>
       <c r="M11" t="n">
         <v>557.2457000000001</v>
       </c>
       <c r="N11" t="n">
-        <v>8.973000000000001</v>
+        <v>0</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>

</xml_diff>